<commit_message>
Updated to reflect psychopy/psychopy@1d7916b4d.b256d5be02db12aa8806ac2ed05f5c54715a2fa2
</commit_message>
<xml_diff>
--- a/psychopy/demos/builder/Experiments/dragAndDrop/stimuli/solutions.xlsx
+++ b/psychopy/demos/builder/Experiments/dragAndDrop/stimuli/solutions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\My Drive\Throwaway\PsychoPy3 Demos\Experiments\dragAndDrop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\psychopy\psychopy\demos\builder\Experiments\dragAndDrop\stimuli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{DCA7A69E-5EAE-4CCD-9941-93DB7F09B9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1355649E-6DD5-4414-88DD-8CD251DE1306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -130,31 +130,31 @@
     <t>pinkSquarePos</t>
   </si>
   <si>
-    <t>(0.2, -0.2)</t>
-  </si>
-  <si>
-    <t>(0, 0.2)</t>
-  </si>
-  <si>
-    <t>(0, -0.2)</t>
-  </si>
-  <si>
-    <t>(0.2, 0.2)</t>
-  </si>
-  <si>
-    <t>(-0.2, -0.2)</t>
-  </si>
-  <si>
-    <t>(-0.2, 0.2)</t>
-  </si>
-  <si>
-    <t>(0.2, 0)</t>
-  </si>
-  <si>
-    <t>(-0.2, 0)</t>
-  </si>
-  <si>
-    <t>(0, 0)</t>
+    <t>[0.2, -0.2]</t>
+  </si>
+  <si>
+    <t>[-0.2, 0.2]</t>
+  </si>
+  <si>
+    <t>[0, -0.2]</t>
+  </si>
+  <si>
+    <t>[-0.2, 0]</t>
+  </si>
+  <si>
+    <t>[0.2, 0.2]</t>
+  </si>
+  <si>
+    <t>[0, 0.2]</t>
+  </si>
+  <si>
+    <t>[-0.2, -0.2]</t>
+  </si>
+  <si>
+    <t>[0, 0]</t>
+  </si>
+  <si>
+    <t>[0.2, 0]</t>
   </si>
 </sst>
 </file>
@@ -563,7 +563,7 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -574,7 +574,7 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
@@ -607,7 +607,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -615,10 +615,10 @@
     </row>
     <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -629,7 +629,7 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
@@ -637,10 +637,10 @@
     </row>
     <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
@@ -651,7 +651,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
         <v>9</v>
@@ -659,10 +659,10 @@
     </row>
     <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>

</xml_diff>